<commit_message>
Add the data-connection rule
A saved query in xl/connections.xml is not an external link: a link reads
cells out of another file, a connection re-runs. Both carry a path, and the
path is the part that outlives the machine. The rule separates a
machine-specific source - a drive letter, a UNC share, an absolute path - from
an https:// one a stranger's copy can still reach.

The dirty fixture gained the part, its content type and its relationship, so
the finding is reproducible from the generator rather than from a binary.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/dirty.xlsx
+++ b/fixtures/dirty.xlsx
@@ -10,6 +10,14 @@
     <definedName name="margin">#REF!</definedName>
   </definedNames>
 </workbook>
+</file>
+
+<file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
+<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <connection id="1" name="RatesTemplate" type="4" refreshedVersion="0" background="1">
+    <webPr xml="1" sourceData="1" url="N:\_Templates\rates\RatesTemplate.xml" htmlTables="1"/>
+  </connection>
+</connections>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>